<commit_message>
Ingest approved entries (2026-09-20)
</commit_message>
<xml_diff>
--- a/candidates/processed/2026-09-14.xlsx
+++ b/candidates/processed/2026-09-14.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
-  <fileVersion appName="Calc" lowestEdited="4"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Candidates" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Lists" sheetId="2" state="hidden" r:id="rId4"/>
+    <sheet name="Candidates" sheetId="1" state="visible" r:id="rId2"/>
+    <sheet name="Lists" sheetId="2" state="hidden" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Candidates!$A$1:$J$1</definedName>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="393" uniqueCount="166">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="398" uniqueCount="166">
   <si>
     <t xml:space="preserve">Include?</t>
   </si>
@@ -89,6 +89,9 @@
     <t xml:space="preserve">https://abcnews.com/Politics/wireStory/federal-judge-freezes-trump-mail-ballot-order-us-136415151</t>
   </si>
   <si>
+    <t xml:space="preserve">Elections</t>
+  </si>
+  <si>
     <t xml:space="preserve">Department of Investigation eyes NYPD disability pensions</t>
   </si>
   <si>
@@ -254,6 +257,9 @@
     <t xml:space="preserve">https://www.npr.org/2026/09/18/g-s1-144112/trump-ban-cnn-msnow-politico-white-house-media</t>
   </si>
   <si>
+    <t xml:space="preserve">Press Freedom</t>
+  </si>
+  <si>
     <t xml:space="preserve">Sep 18</t>
   </si>
   <si>
@@ -299,6 +305,9 @@
     <t xml:space="preserve">https://www.nbcnews.com/politics/trump-administration/trump-announces-agreement-denmark-secure-permanent-control-greenlands-rcna598641</t>
   </si>
   <si>
+    <t xml:space="preserve">Foreign Policy &amp; Aid</t>
+  </si>
+  <si>
     <t xml:space="preserve">California Gov. Gavin Newsom inks AI oversight executive order</t>
   </si>
   <si>
@@ -419,6 +428,9 @@
     <t xml:space="preserve">https://abcnews.com/Politics/wireStory/judge-rules-epa-illegally-terminated-7-billion-solar-136569326</t>
   </si>
   <si>
+    <t xml:space="preserve">Civil Rights &amp; Minorities</t>
+  </si>
+  <si>
     <t xml:space="preserve">Ban on selling handguns to adults under 21 is unconstitutional: Justice Department</t>
   </si>
   <si>
@@ -470,9 +482,6 @@
     <t xml:space="preserve">https://www.pbs.org/newshour/show/u-s-saudi-nuclear-power-deal-faces-pushback-over-potential-weapons-risks</t>
   </si>
   <si>
-    <t xml:space="preserve">Civil Rights &amp; Minorities</t>
-  </si>
-  <si>
     <t xml:space="preserve">Courts &amp; SCOTUS</t>
   </si>
   <si>
@@ -485,9 +494,6 @@
     <t xml:space="preserve">Education</t>
   </si>
   <si>
-    <t xml:space="preserve">Elections</t>
-  </si>
-  <si>
     <t xml:space="preserve">Environment &amp; Science</t>
   </si>
   <si>
@@ -497,9 +503,6 @@
     <t xml:space="preserve">Federal Workforce</t>
   </si>
   <si>
-    <t xml:space="preserve">Foreign Policy &amp; Aid</t>
-  </si>
-  <si>
     <t xml:space="preserve">Free Speech</t>
   </si>
   <si>
@@ -516,9 +519,6 @@
   </si>
   <si>
     <t xml:space="preserve">National Security</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Press Freedom</t>
   </si>
   <si>
     <t xml:space="preserve">Public Health</t>
@@ -534,7 +534,7 @@
   <fonts count="7">
     <font>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
@@ -665,7 +665,6 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FF1F3864"/>
-          <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -673,7 +672,6 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFFFFFFF"/>
-          <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -752,198 +750,23 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
 </file>
 
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
-  <a:themeElements>
-    <a:clrScheme name="Office">
-      <a:dk1>
-        <a:srgbClr val="000000"/>
-      </a:dk1>
-      <a:lt1>
-        <a:srgbClr val="FFFFFF"/>
-      </a:lt1>
-      <a:dk2>
-        <a:srgbClr val="1F497D"/>
-      </a:dk2>
-      <a:lt2>
-        <a:srgbClr val="EEECE1"/>
-      </a:lt2>
-      <a:accent1>
-        <a:srgbClr val="4F81BD"/>
-      </a:accent1>
-      <a:accent2>
-        <a:srgbClr val="C0504D"/>
-      </a:accent2>
-      <a:accent3>
-        <a:srgbClr val="9BBB59"/>
-      </a:accent3>
-      <a:accent4>
-        <a:srgbClr val="8064A2"/>
-      </a:accent4>
-      <a:accent5>
-        <a:srgbClr val="4BACC6"/>
-      </a:accent5>
-      <a:accent6>
-        <a:srgbClr val="F79646"/>
-      </a:accent6>
-      <a:hlink>
-        <a:srgbClr val="0000FF"/>
-      </a:hlink>
-      <a:folHlink>
-        <a:srgbClr val="800080"/>
-      </a:folHlink>
-    </a:clrScheme>
-    <a:fontScheme name="Office">
-      <a:majorFont>
-        <a:latin typeface="Cambria" pitchFamily="0" charset="1"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-      </a:majorFont>
-      <a:minorFont>
-        <a:latin typeface="Calibri" pitchFamily="0" charset="1"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-      </a:minorFont>
-    </a:fontScheme>
-    <a:fmtScheme>
-      <a:fillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:gradFill>
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="50000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="35000">
-              <a:schemeClr val="phClr">
-                <a:tint val="37000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:tint val="15000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
-        </a:gradFill>
-        <a:gradFill>
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="80000">
-              <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="16200000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
-        </a:gradFill>
-      </a:fillStyleLst>
-      <a:lnStyleLst>
-        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-          <a:prstDash val="solid"/>
-        </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
-          <a:prstDash val="solid"/>
-        </a:ln>
-        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </a:lnStyleLst>
-      <a:effectStyleLst>
-        <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-      </a:effectStyleLst>
-      <a:bgFillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:gradFill>
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="40000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="40000">
-              <a:schemeClr val="phClr">
-                <a:tint val="45000"/>
-                <a:shade val="99000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="20000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
-          </a:path>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
-        </a:gradFill>
-        <a:gradFill>
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="80000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="30000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
-          </a:path>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
-        </a:gradFill>
-      </a:bgFillStyleLst>
-    </a:fmtScheme>
-  </a:themeElements>
-</a:theme>
-</file>
-
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:J61"/>
-  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.55078125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="54.99"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="11.99"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="40"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="26"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="0" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="14.01"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="11.99"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1042,7 +865,9 @@
       <c r="E4" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="F4" s="2"/>
+      <c r="F4" s="2" t="s">
+        <v>21</v>
+      </c>
       <c r="G4" s="2"/>
       <c r="H4" s="2"/>
       <c r="I4" s="2" t="s">
@@ -1055,16 +880,16 @@
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2"/>
       <c r="B5" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>11</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
@@ -1073,22 +898,22 @@
         <v>12</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2"/>
       <c r="B6" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
@@ -1097,22 +922,22 @@
         <v>12</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2"/>
       <c r="B7" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F7" s="2"/>
       <c r="G7" s="2"/>
@@ -1121,22 +946,22 @@
         <v>12</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2"/>
       <c r="B8" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>19</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F8" s="2"/>
       <c r="G8" s="2"/>
@@ -1145,22 +970,22 @@
         <v>12</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2"/>
       <c r="B9" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>19</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F9" s="2"/>
       <c r="G9" s="2"/>
@@ -1169,22 +994,22 @@
         <v>12</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2"/>
       <c r="B10" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>19</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F10" s="2"/>
       <c r="G10" s="2"/>
@@ -1193,22 +1018,22 @@
         <v>12</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2"/>
       <c r="B11" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>19</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F11" s="2"/>
       <c r="G11" s="2"/>
@@ -1217,22 +1042,22 @@
         <v>12</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2"/>
       <c r="B12" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F12" s="2"/>
       <c r="G12" s="2"/>
@@ -1241,22 +1066,22 @@
         <v>12</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2"/>
       <c r="B13" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F13" s="2"/>
       <c r="G13" s="2"/>
@@ -1265,22 +1090,22 @@
         <v>12</v>
       </c>
       <c r="J13" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2"/>
       <c r="B14" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>11</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F14" s="2"/>
       <c r="G14" s="2"/>
@@ -1289,22 +1114,22 @@
         <v>12</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2"/>
       <c r="B15" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F15" s="2"/>
       <c r="G15" s="2"/>
@@ -1313,22 +1138,22 @@
         <v>12</v>
       </c>
       <c r="J15" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2"/>
       <c r="B16" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="F16" s="2"/>
       <c r="G16" s="2"/>
@@ -1337,22 +1162,22 @@
         <v>12</v>
       </c>
       <c r="J16" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2"/>
       <c r="B17" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F17" s="2"/>
       <c r="G17" s="2"/>
@@ -1361,22 +1186,22 @@
         <v>12</v>
       </c>
       <c r="J17" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2"/>
       <c r="B18" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="F18" s="2"/>
       <c r="G18" s="2"/>
@@ -1385,22 +1210,22 @@
         <v>12</v>
       </c>
       <c r="J18" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2"/>
       <c r="B19" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F19" s="2"/>
       <c r="G19" s="2"/>
@@ -1409,22 +1234,22 @@
         <v>12</v>
       </c>
       <c r="J19" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2"/>
       <c r="B20" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F20" s="2"/>
       <c r="G20" s="2"/>
@@ -1433,22 +1258,22 @@
         <v>12</v>
       </c>
       <c r="J20" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2"/>
       <c r="B21" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="F21" s="2"/>
       <c r="G21" s="2"/>
@@ -1457,22 +1282,22 @@
         <v>12</v>
       </c>
       <c r="J21" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2"/>
       <c r="B22" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F22" s="2"/>
       <c r="G22" s="2"/>
@@ -1481,22 +1306,22 @@
         <v>12</v>
       </c>
       <c r="J22" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2"/>
       <c r="B23" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F23" s="2"/>
       <c r="G23" s="2"/>
@@ -1505,22 +1330,22 @@
         <v>12</v>
       </c>
       <c r="J23" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2"/>
       <c r="B24" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C24" s="2" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F24" s="2"/>
       <c r="G24" s="2"/>
@@ -1529,22 +1354,22 @@
         <v>12</v>
       </c>
       <c r="J24" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2"/>
       <c r="B25" s="2" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C25" s="2" t="s">
         <v>19</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="F25" s="2"/>
       <c r="G25" s="2"/>
@@ -1553,7 +1378,7 @@
         <v>12</v>
       </c>
       <c r="J25" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1561,40 +1386,42 @@
         <v>17</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="F26" s="2"/>
+        <v>76</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>77</v>
+      </c>
       <c r="G26" s="2"/>
       <c r="H26" s="2"/>
       <c r="I26" s="2" t="s">
         <v>12</v>
       </c>
       <c r="J26" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2"/>
       <c r="B27" s="2" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="F27" s="2"/>
       <c r="G27" s="2"/>
@@ -1603,22 +1430,22 @@
         <v>12</v>
       </c>
       <c r="J27" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="2"/>
       <c r="B28" s="2" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C28" s="2" t="s">
         <v>11</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="F28" s="2"/>
       <c r="G28" s="2"/>
@@ -1627,22 +1454,22 @@
         <v>12</v>
       </c>
       <c r="J28" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="2"/>
       <c r="B29" s="2" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="F29" s="2"/>
       <c r="G29" s="2"/>
@@ -1651,22 +1478,22 @@
         <v>12</v>
       </c>
       <c r="J29" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="2"/>
       <c r="B30" s="2" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="F30" s="2"/>
       <c r="G30" s="2"/>
@@ -1675,22 +1502,22 @@
         <v>12</v>
       </c>
       <c r="J30" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="2"/>
       <c r="B31" s="2" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="F31" s="2"/>
       <c r="G31" s="2"/>
@@ -1699,22 +1526,22 @@
         <v>12</v>
       </c>
       <c r="J31" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="2"/>
       <c r="B32" s="2" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F32" s="2"/>
       <c r="G32" s="2"/>
@@ -1723,7 +1550,7 @@
         <v>12</v>
       </c>
       <c r="J32" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1731,40 +1558,42 @@
         <v>17</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="F33" s="2"/>
+        <v>92</v>
+      </c>
+      <c r="F33" s="2" t="s">
+        <v>93</v>
+      </c>
       <c r="G33" s="2"/>
       <c r="H33" s="2"/>
       <c r="I33" s="2" t="s">
         <v>12</v>
       </c>
       <c r="J33" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="2"/>
       <c r="B34" s="2" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="F34" s="2"/>
       <c r="G34" s="2"/>
@@ -1773,7 +1602,7 @@
         <v>12</v>
       </c>
       <c r="J34" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1781,40 +1610,42 @@
         <v>17</v>
       </c>
       <c r="B35" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="E35" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="F35" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="C35" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="D35" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="E35" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="F35" s="2"/>
       <c r="G35" s="2"/>
       <c r="H35" s="2"/>
       <c r="I35" s="2" t="s">
         <v>12</v>
       </c>
       <c r="J35" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="2"/>
       <c r="B36" s="2" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="F36" s="2"/>
       <c r="G36" s="2"/>
@@ -1823,22 +1654,22 @@
         <v>12</v>
       </c>
       <c r="J36" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="2"/>
       <c r="B37" s="2" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="F37" s="2"/>
       <c r="G37" s="2"/>
@@ -1847,22 +1678,22 @@
         <v>12</v>
       </c>
       <c r="J37" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="2"/>
       <c r="B38" s="2" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="F38" s="2"/>
       <c r="G38" s="2"/>
@@ -1871,22 +1702,22 @@
         <v>12</v>
       </c>
       <c r="J38" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="2"/>
       <c r="B39" s="2" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="F39" s="2"/>
       <c r="G39" s="2"/>
@@ -1895,22 +1726,22 @@
         <v>12</v>
       </c>
       <c r="J39" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="2"/>
       <c r="B40" s="2" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E40" s="3" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="F40" s="2"/>
       <c r="G40" s="2"/>
@@ -1919,22 +1750,22 @@
         <v>12</v>
       </c>
       <c r="J40" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="2"/>
       <c r="B41" s="2" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E41" s="3" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="F41" s="2"/>
       <c r="G41" s="2"/>
@@ -1943,22 +1774,22 @@
         <v>12</v>
       </c>
       <c r="J41" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="2"/>
       <c r="B42" s="2" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E42" s="3" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="F42" s="2"/>
       <c r="G42" s="2"/>
@@ -1967,22 +1798,22 @@
         <v>12</v>
       </c>
       <c r="J42" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="2"/>
       <c r="B43" s="2" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E43" s="3" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="F43" s="2"/>
       <c r="G43" s="2"/>
@@ -1991,22 +1822,22 @@
         <v>12</v>
       </c>
       <c r="J43" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="2"/>
       <c r="B44" s="2" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E44" s="3" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="F44" s="2"/>
       <c r="G44" s="2"/>
@@ -2015,22 +1846,22 @@
         <v>12</v>
       </c>
       <c r="J44" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="2"/>
       <c r="B45" s="2" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E45" s="3" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="F45" s="2"/>
       <c r="G45" s="2"/>
@@ -2039,22 +1870,22 @@
         <v>12</v>
       </c>
       <c r="J45" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="2"/>
       <c r="B46" s="2" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E46" s="3" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="F46" s="2"/>
       <c r="G46" s="2"/>
@@ -2063,22 +1894,22 @@
         <v>12</v>
       </c>
       <c r="J46" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="2"/>
       <c r="B47" s="2" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E47" s="3" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="F47" s="2"/>
       <c r="G47" s="2"/>
@@ -2087,22 +1918,22 @@
         <v>12</v>
       </c>
       <c r="J47" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="2"/>
       <c r="B48" s="2" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E48" s="3" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="F48" s="2"/>
       <c r="G48" s="2"/>
@@ -2111,22 +1942,22 @@
         <v>12</v>
       </c>
       <c r="J48" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="2"/>
       <c r="B49" s="2" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E49" s="3" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="F49" s="2"/>
       <c r="G49" s="2"/>
@@ -2135,22 +1966,22 @@
         <v>12</v>
       </c>
       <c r="J49" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="2"/>
       <c r="B50" s="2" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E50" s="3" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="F50" s="2"/>
       <c r="G50" s="2"/>
@@ -2159,22 +1990,22 @@
         <v>12</v>
       </c>
       <c r="J50" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="2"/>
       <c r="B51" s="2" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E51" s="3" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="F51" s="2"/>
       <c r="G51" s="2"/>
@@ -2183,22 +2014,22 @@
         <v>12</v>
       </c>
       <c r="J51" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="2"/>
       <c r="B52" s="2" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="C52" s="2" t="s">
         <v>19</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E52" s="3" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="F52" s="2"/>
       <c r="G52" s="2"/>
@@ -2207,7 +2038,7 @@
         <v>12</v>
       </c>
       <c r="J52" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2215,40 +2046,42 @@
         <v>17</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="C53" s="2" t="s">
         <v>19</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E53" s="3" t="s">
-        <v>130</v>
-      </c>
-      <c r="F53" s="2"/>
+        <v>133</v>
+      </c>
+      <c r="F53" s="2" t="s">
+        <v>134</v>
+      </c>
       <c r="G53" s="2"/>
       <c r="H53" s="2"/>
       <c r="I53" s="2" t="s">
         <v>12</v>
       </c>
       <c r="J53" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="2"/>
       <c r="B54" s="2" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="C54" s="2" t="s">
         <v>19</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E54" s="3" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="F54" s="2"/>
       <c r="G54" s="2"/>
@@ -2257,22 +2090,22 @@
         <v>12</v>
       </c>
       <c r="J54" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="2"/>
       <c r="B55" s="2" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="C55" s="2" t="s">
         <v>19</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E55" s="3" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="F55" s="2"/>
       <c r="G55" s="2"/>
@@ -2281,22 +2114,22 @@
         <v>12</v>
       </c>
       <c r="J55" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="2"/>
       <c r="B56" s="2" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="C56" s="2" t="s">
         <v>19</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E56" s="3" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="F56" s="2"/>
       <c r="G56" s="2"/>
@@ -2305,22 +2138,22 @@
         <v>12</v>
       </c>
       <c r="J56" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="2"/>
       <c r="B57" s="2" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E57" s="3" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="F57" s="2"/>
       <c r="G57" s="2"/>
@@ -2329,22 +2162,22 @@
         <v>12</v>
       </c>
       <c r="J57" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="2"/>
       <c r="B58" s="2" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E58" s="3" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="F58" s="2"/>
       <c r="G58" s="2"/>
@@ -2353,22 +2186,22 @@
         <v>12</v>
       </c>
       <c r="J58" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="2"/>
       <c r="B59" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="C59" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="C59" s="2" t="s">
-        <v>138</v>
-      </c>
       <c r="D59" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E59" s="3" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="F59" s="2"/>
       <c r="G59" s="2"/>
@@ -2377,22 +2210,22 @@
         <v>12</v>
       </c>
       <c r="J59" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="2"/>
       <c r="B60" s="2" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E60" s="3" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="F60" s="2"/>
       <c r="G60" s="2"/>
@@ -2401,22 +2234,22 @@
         <v>12</v>
       </c>
       <c r="J60" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="2"/>
       <c r="B61" s="2" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E61" s="3" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="F61" s="2"/>
       <c r="G61" s="2"/>
@@ -2425,7 +2258,7 @@
         <v>12</v>
       </c>
       <c r="J61" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
   </sheetData>
@@ -2519,96 +2352,96 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:A18"/>
-  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.55078125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
-        <v>148</v>
+        <v>134</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>153</v>
+        <v>21</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>157</v>
+        <v>93</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="0" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="0" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="0" t="s">
-        <v>164</v>
+        <v>77</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>